<commit_message>
prepare to June with Lab
</commit_message>
<xml_diff>
--- a/Data/Meansurement.xlsx
+++ b/Data/Meansurement.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Senior Project\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0077093C-70D2-4D9F-A7A5-8549943B74DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47112E87-AAC3-4DDF-A774-7040541B1F08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hourly Room Temp" sheetId="1" r:id="rId1"/>
@@ -22391,15 +22391,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101004A83FCAD2B02494AB70746B544CC61AE" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="77bfa71e1908209a377d80d9948cd243">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="228fa7ca-c38f-4560-861c-8ff0895b344f" xmlns:ns3="60441c17-193d-4aaa-84fe-076df351db0c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cf08252bb5eb797fcd948f11b977b465" ns2:_="" ns3:_="">
     <xsd:import namespace="228fa7ca-c38f-4560-861c-8ff0895b344f"/>
@@ -22588,6 +22579,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBA7AD0B-D9B0-45DE-A7AE-8A303D13225D}">
   <ds:schemaRefs>
@@ -22600,14 +22600,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{94823659-B512-4ECA-9D86-4915201F8F7B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D94FF3E2-982E-40E4-B192-D71C6EF31E2D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -22624,4 +22616,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{94823659-B512-4ECA-9D86-4915201F8F7B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>